<commit_message>
fix for the template
</commit_message>
<xml_diff>
--- a/api/templates/all_results/es.xlsx
+++ b/api/templates/all_results/es.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24701"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\ubuntu\aspect\api\templates\export\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\ubuntu\aspect\api\templates\all_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F156F1-525D-4589-96F2-EB33BEDC1B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E2F239E-A1F1-48A6-8835-C7CCC53EFBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21220" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -151,9 +151,6 @@
     <t>Resultados</t>
   </si>
   <si>
-    <t>Impreso &lt;date&gt;</t>
-  </si>
-  <si>
     <t>Día del test</t>
   </si>
   <si>
@@ -203,6 +200,9 @@
   </si>
   <si>
     <t>Sitio</t>
+  </si>
+  <si>
+    <t>Impreso &lt;Dates&gt;</t>
   </si>
 </sst>
 </file>
@@ -874,7 +874,7 @@
     </row>
     <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8"/>
@@ -909,46 +909,46 @@
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="23"/>
       <c r="E5" s="23"/>
       <c r="F5" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="G5" s="20" t="s">
-        <v>50</v>
-      </c>
       <c r="H5" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I5" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="J5" s="20" t="s">
-        <v>54</v>
-      </c>
       <c r="K5" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="23"/>
       <c r="B6" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="D6" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>44</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>45</v>
       </c>
       <c r="F6" s="21"/>
       <c r="G6" s="21"/>
@@ -974,19 +974,19 @@
         <v>38</v>
       </c>
       <c r="F7" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="G7" s="11" t="s">
-        <v>48</v>
-      </c>
       <c r="H7" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I7" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" s="17" t="s">
         <v>51</v>
-      </c>
-      <c r="J7" s="17" t="s">
-        <v>52</v>
       </c>
       <c r="K7" s="12" t="s">
         <v>39</v>

</xml_diff>